<commit_message>
Update all code: registration, admin commands, tracking
</commit_message>
<xml_diff>
--- a/Order 1.24.2026 .xlsx
+++ b/Order 1.24.2026 .xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\muslat_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD6BF34-6CDA-44B7-AC3F-0E93809A37D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45943B4B-70E3-4275-B97E-968C52ABFB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{82A12A56-94C1-4E1B-81BF-390885B4DE72}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{82A12A56-94C1-4E1B-81BF-390885B4DE72}"/>
   </bookViews>
   <sheets>
     <sheet name="CLEAN_DATA" sheetId="21" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="22" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="342">
   <si>
     <t>Nodira</t>
   </si>
@@ -1044,6 +1045,27 @@
   </si>
   <si>
     <t>YT8834523358954</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Packed</t>
+  </si>
+  <si>
+    <t>In Transit</t>
+  </si>
+  <si>
+    <t>Arrived</t>
+  </si>
+  <si>
+    <t>Last Mile</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received </t>
   </si>
 </sst>
 </file>
@@ -1439,15 +1461,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C79EED2-BB45-4DCE-98C8-7C19777A94D8}">
-  <dimension ref="A1:C274"/>
+  <dimension ref="A1:D274"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" customWidth="1"/>
     <col min="2" max="2" width="29.5703125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>331</v>
       </c>
@@ -1457,8 +1480,11 @@
       <c r="C1" s="1" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>228</v>
       </c>
@@ -1468,8 +1494,11 @@
       <c r="C2" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>229</v>
       </c>
@@ -1479,8 +1508,11 @@
       <c r="C3" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>230</v>
       </c>
@@ -1490,8 +1522,11 @@
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>231</v>
       </c>
@@ -1501,8 +1536,11 @@
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>232</v>
       </c>
@@ -1512,8 +1550,11 @@
       <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>233</v>
       </c>
@@ -1523,8 +1564,11 @@
       <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>234</v>
       </c>
@@ -1534,8 +1578,11 @@
       <c r="C8" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>235</v>
       </c>
@@ -1545,8 +1592,11 @@
       <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>236</v>
       </c>
@@ -1556,8 +1606,11 @@
       <c r="C10" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>237</v>
       </c>
@@ -1567,8 +1620,11 @@
       <c r="C11" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>238</v>
       </c>
@@ -1578,8 +1634,11 @@
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>239</v>
       </c>
@@ -1589,8 +1648,11 @@
       <c r="C13" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>240</v>
       </c>
@@ -1600,8 +1662,11 @@
       <c r="C14" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>241</v>
       </c>
@@ -1611,8 +1676,11 @@
       <c r="C15" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>242</v>
       </c>
@@ -1622,8 +1690,11 @@
       <c r="C16" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>243</v>
       </c>
@@ -1633,8 +1704,11 @@
       <c r="C17" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>244</v>
       </c>
@@ -1644,8 +1718,11 @@
       <c r="C18" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>245</v>
       </c>
@@ -1655,8 +1732,11 @@
       <c r="C19" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>246</v>
       </c>
@@ -1666,8 +1746,11 @@
       <c r="C20" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>247</v>
       </c>
@@ -1677,8 +1760,11 @@
       <c r="C21" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>248</v>
       </c>
@@ -1688,8 +1774,11 @@
       <c r="C22" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>249</v>
       </c>
@@ -1699,8 +1788,11 @@
       <c r="C23" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>250</v>
       </c>
@@ -1710,8 +1802,11 @@
       <c r="C24" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>251</v>
       </c>
@@ -1721,8 +1816,11 @@
       <c r="C25" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>252</v>
       </c>
@@ -1732,8 +1830,11 @@
       <c r="C26" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>253</v>
       </c>
@@ -1743,8 +1844,11 @@
       <c r="C27" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>254</v>
       </c>
@@ -1754,8 +1858,11 @@
       <c r="C28" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>255</v>
       </c>
@@ -1765,8 +1872,11 @@
       <c r="C29" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>256</v>
       </c>
@@ -1776,8 +1886,11 @@
       <c r="C30" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>257</v>
       </c>
@@ -1787,8 +1900,11 @@
       <c r="C31" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>258</v>
       </c>
@@ -1798,8 +1914,11 @@
       <c r="C32" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>276</v>
       </c>
@@ -1809,8 +1928,11 @@
       <c r="C33" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>259</v>
       </c>
@@ -1820,8 +1942,11 @@
       <c r="C34" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>260</v>
       </c>
@@ -1831,8 +1956,11 @@
       <c r="C35" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>261</v>
       </c>
@@ -1842,8 +1970,11 @@
       <c r="C36" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D36" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>262</v>
       </c>
@@ -1853,8 +1984,11 @@
       <c r="C37" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>263</v>
       </c>
@@ -1864,8 +1998,11 @@
       <c r="C38" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>264</v>
       </c>
@@ -1875,8 +2012,11 @@
       <c r="C39" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>265</v>
       </c>
@@ -1886,8 +2026,11 @@
       <c r="C40" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>266</v>
       </c>
@@ -1897,8 +2040,11 @@
       <c r="C41" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>267</v>
       </c>
@@ -1908,8 +2054,11 @@
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>268</v>
       </c>
@@ -1919,8 +2068,11 @@
       <c r="C43" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>269</v>
       </c>
@@ -1930,8 +2082,11 @@
       <c r="C44" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D44" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>270</v>
       </c>
@@ -1941,8 +2096,11 @@
       <c r="C45" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>271</v>
       </c>
@@ -1952,8 +2110,11 @@
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D46" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>272</v>
       </c>
@@ -1963,8 +2124,11 @@
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>273</v>
       </c>
@@ -1974,8 +2138,11 @@
       <c r="C48" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>274</v>
       </c>
@@ -1985,8 +2152,11 @@
       <c r="C49" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>275</v>
       </c>
@@ -1996,8 +2166,11 @@
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>277</v>
       </c>
@@ -2007,8 +2180,11 @@
       <c r="C51" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D51" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>278</v>
       </c>
@@ -2018,8 +2194,11 @@
       <c r="C52" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>279</v>
       </c>
@@ -2029,8 +2208,11 @@
       <c r="C53" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>280</v>
       </c>
@@ -2040,8 +2222,11 @@
       <c r="C54" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>281</v>
       </c>
@@ -2051,8 +2236,11 @@
       <c r="C55" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D55" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>282</v>
       </c>
@@ -2062,8 +2250,11 @@
       <c r="C56" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D56" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>283</v>
       </c>
@@ -2073,8 +2264,11 @@
       <c r="C57" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D57" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>284</v>
       </c>
@@ -2084,8 +2278,11 @@
       <c r="C58" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D58" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>285</v>
       </c>
@@ -2095,8 +2292,11 @@
       <c r="C59" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D59" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>286</v>
       </c>
@@ -2106,8 +2306,11 @@
       <c r="C60" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D60" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>287</v>
       </c>
@@ -2117,8 +2320,11 @@
       <c r="C61" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D61" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>288</v>
       </c>
@@ -2128,8 +2334,11 @@
       <c r="C62" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D62" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>289</v>
       </c>
@@ -2139,8 +2348,11 @@
       <c r="C63" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D63" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>290</v>
       </c>
@@ -2150,8 +2362,11 @@
       <c r="C64" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D64" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>291</v>
       </c>
@@ -2161,8 +2376,11 @@
       <c r="C65" s="3" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>292</v>
       </c>
@@ -2172,8 +2390,11 @@
       <c r="C66" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D66" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>293</v>
       </c>
@@ -2183,8 +2404,11 @@
       <c r="C67" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D67" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>294</v>
       </c>
@@ -2194,8 +2418,11 @@
       <c r="C68" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D68" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>295</v>
       </c>
@@ -2205,8 +2432,11 @@
       <c r="C69" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D69" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>296</v>
       </c>
@@ -2216,8 +2446,11 @@
       <c r="C70" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D70" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>297</v>
       </c>
@@ -2227,8 +2460,11 @@
       <c r="C71" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D71" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>298</v>
       </c>
@@ -2238,8 +2474,11 @@
       <c r="C72" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D72" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>299</v>
       </c>
@@ -2249,8 +2488,11 @@
       <c r="C73" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D73" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>300</v>
       </c>
@@ -2260,8 +2502,11 @@
       <c r="C74" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D74" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>301</v>
       </c>
@@ -2271,8 +2516,11 @@
       <c r="C75" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D75" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>302</v>
       </c>
@@ -2282,8 +2530,11 @@
       <c r="C76" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>303</v>
       </c>
@@ -2293,8 +2544,11 @@
       <c r="C77" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D77" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>304</v>
       </c>
@@ -2304,8 +2558,11 @@
       <c r="C78" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D78" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>305</v>
       </c>
@@ -2315,8 +2572,11 @@
       <c r="C79" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D79" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>306</v>
       </c>
@@ -2326,8 +2586,11 @@
       <c r="C80" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>307</v>
       </c>
@@ -2337,8 +2600,11 @@
       <c r="C81" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D81" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>308</v>
       </c>
@@ -2348,8 +2614,11 @@
       <c r="C82" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D82" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>309</v>
       </c>
@@ -2359,8 +2628,11 @@
       <c r="C83" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>310</v>
       </c>
@@ -2370,8 +2642,11 @@
       <c r="C84" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D84" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>311</v>
       </c>
@@ -2381,8 +2656,11 @@
       <c r="C85" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D85" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>312</v>
       </c>
@@ -2392,8 +2670,11 @@
       <c r="C86" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>313</v>
       </c>
@@ -2403,8 +2684,11 @@
       <c r="C87" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D87" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>314</v>
       </c>
@@ -2414,8 +2698,11 @@
       <c r="C88" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>315</v>
       </c>
@@ -2425,8 +2712,11 @@
       <c r="C89" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>316</v>
       </c>
@@ -2436,8 +2726,11 @@
       <c r="C90" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D90" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>317</v>
       </c>
@@ -2447,8 +2740,11 @@
       <c r="C91" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D91" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>318</v>
       </c>
@@ -2458,8 +2754,11 @@
       <c r="C92" s="3" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D92" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>319</v>
       </c>
@@ -2469,8 +2768,11 @@
       <c r="C93" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D93" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>320</v>
       </c>
@@ -2480,8 +2782,11 @@
       <c r="C94" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D94" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>321</v>
       </c>
@@ -2491,8 +2796,11 @@
       <c r="C95" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D95" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>322</v>
       </c>
@@ -2502,8 +2810,11 @@
       <c r="C96" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D96" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>323</v>
       </c>
@@ -2513,8 +2824,11 @@
       <c r="C97" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D97" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>324</v>
       </c>
@@ -2524,8 +2838,11 @@
       <c r="C98" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D98" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>58</v>
       </c>
@@ -2535,8 +2852,11 @@
       <c r="C99" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D99" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>59</v>
       </c>
@@ -2546,8 +2866,11 @@
       <c r="C100" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D100" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>65</v>
       </c>
@@ -2557,8 +2880,11 @@
       <c r="C101" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>64</v>
       </c>
@@ -2568,8 +2894,11 @@
       <c r="C102" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D102" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>63</v>
       </c>
@@ -2579,8 +2908,11 @@
       <c r="C103" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D103" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>75</v>
       </c>
@@ -2590,8 +2922,11 @@
       <c r="C104" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D104" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>66</v>
       </c>
@@ -2601,8 +2936,11 @@
       <c r="C105" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D105" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>67</v>
       </c>
@@ -2612,8 +2950,11 @@
       <c r="C106" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D106" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>68</v>
       </c>
@@ -2623,8 +2964,11 @@
       <c r="C107" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D107" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>66</v>
       </c>
@@ -2634,8 +2978,11 @@
       <c r="C108" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D108" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>60</v>
       </c>
@@ -2645,8 +2992,11 @@
       <c r="C109" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D109" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>61</v>
       </c>
@@ -2656,8 +3006,11 @@
       <c r="C110" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D110" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>62</v>
       </c>
@@ -2667,8 +3020,11 @@
       <c r="C111" s="2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D111" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>70</v>
       </c>
@@ -2678,8 +3034,11 @@
       <c r="C112" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D112" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>71</v>
       </c>
@@ -2689,8 +3048,11 @@
       <c r="C113" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D113" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>74</v>
       </c>
@@ -2700,8 +3062,11 @@
       <c r="C114" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D114" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>76</v>
       </c>
@@ -2711,8 +3076,11 @@
       <c r="C115" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>77</v>
       </c>
@@ -2722,8 +3090,11 @@
       <c r="C116" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>78</v>
       </c>
@@ -2733,8 +3104,11 @@
       <c r="C117" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D117" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>79</v>
       </c>
@@ -2744,8 +3118,11 @@
       <c r="C118" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D118" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>82</v>
       </c>
@@ -2755,8 +3132,11 @@
       <c r="C119" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D119" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>83</v>
       </c>
@@ -2766,8 +3146,11 @@
       <c r="C120" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D120" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>85</v>
       </c>
@@ -2777,8 +3160,11 @@
       <c r="C121" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D121" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>87</v>
       </c>
@@ -2788,8 +3174,11 @@
       <c r="C122" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D122" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>90</v>
       </c>
@@ -2799,8 +3188,11 @@
       <c r="C123" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D123" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>92</v>
       </c>
@@ -2810,8 +3202,11 @@
       <c r="C124" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D124" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>93</v>
       </c>
@@ -2821,8 +3216,11 @@
       <c r="C125" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D125" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>94</v>
       </c>
@@ -2832,8 +3230,11 @@
       <c r="C126" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D126" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>97</v>
       </c>
@@ -2843,8 +3244,11 @@
       <c r="C127" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D127" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>98</v>
       </c>
@@ -2854,8 +3258,11 @@
       <c r="C128" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D128" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
         <v>99</v>
       </c>
@@ -2865,8 +3272,11 @@
       <c r="C129" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D129" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
         <v>100</v>
       </c>
@@ -2876,8 +3286,11 @@
       <c r="C130" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D130" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
         <v>101</v>
       </c>
@@ -2887,8 +3300,11 @@
       <c r="C131" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D131" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>102</v>
       </c>
@@ -2898,8 +3314,11 @@
       <c r="C132" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>105</v>
       </c>
@@ -2909,8 +3328,11 @@
       <c r="C133" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D133" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
         <v>106</v>
       </c>
@@ -2920,8 +3342,11 @@
       <c r="C134" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>107</v>
       </c>
@@ -2931,8 +3356,11 @@
       <c r="C135" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D135" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>108</v>
       </c>
@@ -2942,8 +3370,11 @@
       <c r="C136" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D136" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>109</v>
       </c>
@@ -2953,8 +3384,11 @@
       <c r="C137" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D137" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>110</v>
       </c>
@@ -2964,8 +3398,11 @@
       <c r="C138" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D138" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
         <v>111</v>
       </c>
@@ -2975,8 +3412,11 @@
       <c r="C139" s="3" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D139" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
         <v>122</v>
       </c>
@@ -2986,8 +3426,11 @@
       <c r="C140" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D140" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>114</v>
       </c>
@@ -2997,8 +3440,11 @@
       <c r="C141" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D141" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>115</v>
       </c>
@@ -3008,8 +3454,11 @@
       <c r="C142" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D142" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>116</v>
       </c>
@@ -3019,8 +3468,11 @@
       <c r="C143" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D143" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
         <v>119</v>
       </c>
@@ -3030,8 +3482,11 @@
       <c r="C144" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D144" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
         <v>120</v>
       </c>
@@ -3041,8 +3496,11 @@
       <c r="C145" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D145" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
         <v>121</v>
       </c>
@@ -3052,8 +3510,11 @@
       <c r="C146" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D146" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>123</v>
       </c>
@@ -3063,8 +3524,11 @@
       <c r="C147" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D147" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>124</v>
       </c>
@@ -3074,8 +3538,11 @@
       <c r="C148" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D148" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
         <v>125</v>
       </c>
@@ -3085,8 +3552,11 @@
       <c r="C149" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D149" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
         <v>126</v>
       </c>
@@ -3096,8 +3566,11 @@
       <c r="C150" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D150" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
         <v>127</v>
       </c>
@@ -3107,8 +3580,11 @@
       <c r="C151" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D151" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
         <v>128</v>
       </c>
@@ -3118,8 +3594,11 @@
       <c r="C152" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D152" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
         <v>129</v>
       </c>
@@ -3129,8 +3608,11 @@
       <c r="C153" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D153" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
         <v>130</v>
       </c>
@@ -3140,8 +3622,11 @@
       <c r="C154" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D154" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
         <v>136</v>
       </c>
@@ -3151,8 +3636,11 @@
       <c r="C155" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D155" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
         <v>131</v>
       </c>
@@ -3162,8 +3650,11 @@
       <c r="C156" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D156" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
         <v>132</v>
       </c>
@@ -3173,8 +3664,11 @@
       <c r="C157" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D157" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
         <v>133</v>
       </c>
@@ -3184,8 +3678,11 @@
       <c r="C158" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D158" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="3" t="s">
         <v>134</v>
       </c>
@@ -3195,8 +3692,11 @@
       <c r="C159" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D159" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="3" t="s">
         <v>135</v>
       </c>
@@ -3206,8 +3706,11 @@
       <c r="C160" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D160" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
         <v>137</v>
       </c>
@@ -3217,8 +3720,11 @@
       <c r="C161" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D161" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
         <v>139</v>
       </c>
@@ -3228,8 +3734,11 @@
       <c r="C162" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D162" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
         <v>138</v>
       </c>
@@ -3239,8 +3748,11 @@
       <c r="C163" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D163" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
         <v>142</v>
       </c>
@@ -3250,8 +3762,11 @@
       <c r="C164" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D164" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
         <v>143</v>
       </c>
@@ -3261,8 +3776,11 @@
       <c r="C165" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D165" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
         <v>144</v>
       </c>
@@ -3272,8 +3790,11 @@
       <c r="C166" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D166" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
         <v>159</v>
       </c>
@@ -3283,8 +3804,11 @@
       <c r="C167" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D167" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
         <v>145</v>
       </c>
@@ -3294,8 +3818,11 @@
       <c r="C168" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D168" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
         <v>153</v>
       </c>
@@ -3305,8 +3832,11 @@
       <c r="C169" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D169" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>152</v>
       </c>
@@ -3316,8 +3846,11 @@
       <c r="C170" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D170" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
         <v>150</v>
       </c>
@@ -3327,8 +3860,11 @@
       <c r="C171" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D171" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
         <v>147</v>
       </c>
@@ -3338,8 +3874,11 @@
       <c r="C172" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D172" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>148</v>
       </c>
@@ -3349,8 +3888,11 @@
       <c r="C173" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D173" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="3" t="s">
         <v>149</v>
       </c>
@@ -3360,8 +3902,11 @@
       <c r="C174" s="3" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D174" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="s">
         <v>157</v>
       </c>
@@ -3371,8 +3916,11 @@
       <c r="C175" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D175" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="s">
         <v>151</v>
       </c>
@@ -3382,8 +3930,11 @@
       <c r="C176" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D176" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
         <v>156</v>
       </c>
@@ -3393,8 +3944,11 @@
       <c r="C177" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D177" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
         <v>154</v>
       </c>
@@ -3404,8 +3958,11 @@
       <c r="C178" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D178" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
         <v>155</v>
       </c>
@@ -3415,8 +3972,11 @@
       <c r="C179" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D179" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
         <v>158</v>
       </c>
@@ -3426,8 +3986,11 @@
       <c r="C180" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D180" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
         <v>160</v>
       </c>
@@ -3437,8 +4000,11 @@
       <c r="C181" s="2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D181" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
         <v>161</v>
       </c>
@@ -3448,8 +4014,11 @@
       <c r="C182" s="2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D182" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
         <v>162</v>
       </c>
@@ -3459,8 +4028,11 @@
       <c r="C183" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D183" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
         <v>163</v>
       </c>
@@ -3470,8 +4042,11 @@
       <c r="C184" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D184" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
         <v>164</v>
       </c>
@@ -3481,8 +4056,11 @@
       <c r="C185" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D185" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
         <v>165</v>
       </c>
@@ -3492,8 +4070,11 @@
       <c r="C186" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D186" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
         <v>166</v>
       </c>
@@ -3503,8 +4084,11 @@
       <c r="C187" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D187" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
         <v>167</v>
       </c>
@@ -3514,8 +4098,11 @@
       <c r="C188" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D188" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="3" t="s">
         <v>168</v>
       </c>
@@ -3525,8 +4112,11 @@
       <c r="C189" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D189" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
         <v>169</v>
       </c>
@@ -3536,8 +4126,11 @@
       <c r="C190" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D190" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
         <v>170</v>
       </c>
@@ -3547,8 +4140,11 @@
       <c r="C191" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D191" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
         <v>171</v>
       </c>
@@ -3558,8 +4154,11 @@
       <c r="C192" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D192" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="3" t="s">
         <v>172</v>
       </c>
@@ -3569,8 +4168,11 @@
       <c r="C193" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D193" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="3" t="s">
         <v>173</v>
       </c>
@@ -3580,8 +4182,11 @@
       <c r="C194" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D194" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
         <v>174</v>
       </c>
@@ -3591,8 +4196,11 @@
       <c r="C195" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D195" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
         <v>175</v>
       </c>
@@ -3602,8 +4210,11 @@
       <c r="C196" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D196" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="3" t="s">
         <v>176</v>
       </c>
@@ -3613,8 +4224,11 @@
       <c r="C197" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D197" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>177</v>
       </c>
@@ -3624,8 +4238,11 @@
       <c r="C198" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D198" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>178</v>
       </c>
@@ -3635,8 +4252,11 @@
       <c r="C199" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D199" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>179</v>
       </c>
@@ -3646,8 +4266,11 @@
       <c r="C200" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D200" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>180</v>
       </c>
@@ -3657,8 +4280,11 @@
       <c r="C201" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D201" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="3" t="s">
         <v>190</v>
       </c>
@@ -3668,8 +4294,11 @@
       <c r="C202" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D202" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="3" t="s">
         <v>189</v>
       </c>
@@ -3679,8 +4308,11 @@
       <c r="C203" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D203" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>181</v>
       </c>
@@ -3690,8 +4322,11 @@
       <c r="C204" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D204" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>183</v>
       </c>
@@ -3701,8 +4336,11 @@
       <c r="C205" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D205" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>182</v>
       </c>
@@ -3712,8 +4350,11 @@
       <c r="C206" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D206" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>183</v>
       </c>
@@ -3723,8 +4364,11 @@
       <c r="C207" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D207" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>184</v>
       </c>
@@ -3734,8 +4378,11 @@
       <c r="C208" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D208" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>185</v>
       </c>
@@ -3745,8 +4392,11 @@
       <c r="C209" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D209" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>186</v>
       </c>
@@ -3756,8 +4406,11 @@
       <c r="C210" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D210" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>187</v>
       </c>
@@ -3767,8 +4420,11 @@
       <c r="C211" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D211" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>202</v>
       </c>
@@ -3778,8 +4434,11 @@
       <c r="C212" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D212" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>201</v>
       </c>
@@ -3789,8 +4448,11 @@
       <c r="C213" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D213" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" s="3" t="s">
         <v>188</v>
       </c>
@@ -3800,8 +4462,11 @@
       <c r="C214" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D214" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" s="3" t="s">
         <v>191</v>
       </c>
@@ -3811,8 +4476,11 @@
       <c r="C215" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D215" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
         <v>194</v>
       </c>
@@ -3822,8 +4490,11 @@
       <c r="C216" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D216" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="3" t="s">
         <v>195</v>
       </c>
@@ -3833,8 +4504,11 @@
       <c r="C217" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D217" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="3" t="s">
         <v>203</v>
       </c>
@@ -3844,8 +4518,11 @@
       <c r="C218" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D218" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" s="3" t="s">
         <v>199</v>
       </c>
@@ -3855,8 +4532,11 @@
       <c r="C219" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D219" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" s="3" t="s">
         <v>196</v>
       </c>
@@ -3866,8 +4546,11 @@
       <c r="C220" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D220" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" s="3" t="s">
         <v>197</v>
       </c>
@@ -3877,8 +4560,11 @@
       <c r="C221" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D221" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="3" t="s">
         <v>204</v>
       </c>
@@ -3888,8 +4574,11 @@
       <c r="C222" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D222" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" s="3" t="s">
         <v>198</v>
       </c>
@@ -3899,8 +4588,11 @@
       <c r="C223" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D223" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" s="3" t="s">
         <v>200</v>
       </c>
@@ -3910,8 +4602,11 @@
       <c r="C224" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D224" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" s="3" t="s">
         <v>25</v>
       </c>
@@ -3921,8 +4616,11 @@
       <c r="C225" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D225" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" s="3" t="s">
         <v>35</v>
       </c>
@@ -3932,8 +4630,11 @@
       <c r="C226" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D226" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" s="3" t="s">
         <v>26</v>
       </c>
@@ -3943,8 +4644,11 @@
       <c r="C227" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D227" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" s="3" t="s">
         <v>27</v>
       </c>
@@ -3954,8 +4658,11 @@
       <c r="C228" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D228" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" s="3" t="s">
         <v>43</v>
       </c>
@@ -3965,8 +4672,11 @@
       <c r="C229" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D229" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" s="3" t="s">
         <v>28</v>
       </c>
@@ -3976,8 +4686,11 @@
       <c r="C230" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D230" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" s="3" t="s">
         <v>31</v>
       </c>
@@ -3987,8 +4700,11 @@
       <c r="C231" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D231" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" s="3" t="s">
         <v>34</v>
       </c>
@@ -3998,8 +4714,11 @@
       <c r="C232" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D232" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" s="3" t="s">
         <v>44</v>
       </c>
@@ -4009,8 +4728,11 @@
       <c r="C233" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D233" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
         <v>32</v>
       </c>
@@ -4020,8 +4742,11 @@
       <c r="C234" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D234" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
         <v>39</v>
       </c>
@@ -4031,8 +4756,11 @@
       <c r="C235" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D235" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
         <v>40</v>
       </c>
@@ -4042,8 +4770,11 @@
       <c r="C236" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D236" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
         <v>41</v>
       </c>
@@ -4053,8 +4784,11 @@
       <c r="C237" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D237" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" s="3" t="s">
         <v>42</v>
       </c>
@@ -4064,8 +4798,11 @@
       <c r="C238" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D238" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" s="3" t="s">
         <v>45</v>
       </c>
@@ -4075,8 +4812,11 @@
       <c r="C239" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D239" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" s="3" t="s">
         <v>46</v>
       </c>
@@ -4086,8 +4826,11 @@
       <c r="C240" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D240" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" s="3" t="s">
         <v>33</v>
       </c>
@@ -4097,8 +4840,11 @@
       <c r="C241" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D241" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" s="3" t="s">
         <v>36</v>
       </c>
@@ -4108,8 +4854,11 @@
       <c r="C242" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D242" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" s="3" t="s">
         <v>37</v>
       </c>
@@ -4119,8 +4868,11 @@
       <c r="C243" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D243" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" s="3" t="s">
         <v>38</v>
       </c>
@@ -4130,8 +4882,11 @@
       <c r="C244" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D244" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" s="3" t="s">
         <v>47</v>
       </c>
@@ -4141,8 +4896,11 @@
       <c r="C245" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D245" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" s="3" t="s">
         <v>52</v>
       </c>
@@ -4152,8 +4910,11 @@
       <c r="C246" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D246" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" s="3" t="s">
         <v>48</v>
       </c>
@@ -4163,8 +4924,11 @@
       <c r="C247" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D247" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" s="3" t="s">
         <v>49</v>
       </c>
@@ -4174,8 +4938,11 @@
       <c r="C248" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D248" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" s="3" t="s">
         <v>50</v>
       </c>
@@ -4185,8 +4952,11 @@
       <c r="C249" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D249" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" s="3" t="s">
         <v>51</v>
       </c>
@@ -4196,8 +4966,11 @@
       <c r="C250" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D250" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" s="3" t="s">
         <v>53</v>
       </c>
@@ -4207,8 +4980,11 @@
       <c r="C251" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D251" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" s="3" t="s">
         <v>54</v>
       </c>
@@ -4218,8 +4994,11 @@
       <c r="C252" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D252" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" s="3" t="s">
         <v>55</v>
       </c>
@@ -4229,8 +5008,11 @@
       <c r="C253" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D253" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" s="3" t="s">
         <v>205</v>
       </c>
@@ -4240,8 +5022,11 @@
       <c r="C254" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D254" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" s="3" t="s">
         <v>220</v>
       </c>
@@ -4251,8 +5036,11 @@
       <c r="C255" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D255" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" s="3" t="s">
         <v>218</v>
       </c>
@@ -4262,8 +5050,11 @@
       <c r="C256" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D256" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
         <v>208</v>
       </c>
@@ -4273,8 +5064,11 @@
       <c r="C257" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D257" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" s="3" t="s">
         <v>207</v>
       </c>
@@ -4284,8 +5078,11 @@
       <c r="C258" s="3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D258" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" s="3" t="s">
         <v>225</v>
       </c>
@@ -4295,8 +5092,11 @@
       <c r="C259" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D259" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
         <v>214</v>
       </c>
@@ -4306,8 +5106,11 @@
       <c r="C260" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D260" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
         <v>209</v>
       </c>
@@ -4317,8 +5120,11 @@
       <c r="C261" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D261" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
         <v>210</v>
       </c>
@@ -4328,8 +5134,11 @@
       <c r="C262" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D262" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
         <v>222</v>
       </c>
@@ -4339,8 +5148,11 @@
       <c r="C263" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D263" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
         <v>211</v>
       </c>
@@ -4350,8 +5162,11 @@
       <c r="C264" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D264" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
         <v>212</v>
       </c>
@@ -4361,8 +5176,11 @@
       <c r="C265" s="3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D265" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="3" t="s">
         <v>217</v>
       </c>
@@ -4372,8 +5190,11 @@
       <c r="C266" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D266" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
         <v>216</v>
       </c>
@@ -4383,8 +5204,11 @@
       <c r="C267" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D267" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="3" t="s">
         <v>213</v>
       </c>
@@ -4394,8 +5218,11 @@
       <c r="C268" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D268" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" s="3" t="s">
         <v>334</v>
       </c>
@@ -4405,8 +5232,11 @@
       <c r="C269" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D269" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" s="3" t="s">
         <v>221</v>
       </c>
@@ -4416,8 +5246,11 @@
       <c r="C270" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D270" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" s="3" t="s">
         <v>215</v>
       </c>
@@ -4427,8 +5260,11 @@
       <c r="C271" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D271" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" s="3" t="s">
         <v>219</v>
       </c>
@@ -4438,8 +5274,11 @@
       <c r="C272" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D272" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" s="3" t="s">
         <v>223</v>
       </c>
@@ -4449,8 +5288,11 @@
       <c r="C273" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D273" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" s="3" t="s">
         <v>224</v>
       </c>
@@ -4459,6 +5301,65 @@
       </c>
       <c r="C274" s="3" t="s">
         <v>57</v>
+      </c>
+      <c r="D274" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataConsolidate/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0FF2C097-D524-4CB6-B4FD-1CF881695EC4}">
+          <x14:formula1>
+            <xm:f>Sheet1!$A$1:$A$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D274</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27671C38-AFD6-44F2-83C1-4A64B8720F6F}">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Delete old database file on startup
</commit_message>
<xml_diff>
--- a/Order 1.24.2026 .xlsx
+++ b/Order 1.24.2026 .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\muslat_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45943B4B-70E3-4275-B97E-968C52ABFB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B597FA33-3A82-40DB-9756-DF018AEBC7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{82A12A56-94C1-4E1B-81BF-390885B4DE72}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{82A12A56-94C1-4E1B-81BF-390885B4DE72}"/>
   </bookViews>
   <sheets>
     <sheet name="CLEAN_DATA" sheetId="21" r:id="rId1"/>
@@ -1461,16 +1461,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C79EED2-BB45-4DCE-98C8-7C19777A94D8}">
-  <dimension ref="A1:D274"/>
+  <dimension ref="A1:E274"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" customWidth="1"/>
     <col min="2" max="2" width="29.5703125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>331</v>
       </c>
@@ -1484,7 +1485,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>228</v>
       </c>
@@ -1497,8 +1498,12 @@
       <c r="D2" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="str">
+        <f xml:space="preserve"> "/addshipment "&amp;A2&amp;" "&amp;B2&amp;" "&amp;C2&amp;" "&amp;D2</f>
+        <v>/addshipment YT88311855941829 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>229</v>
       </c>
@@ -1511,8 +1516,12 @@
       <c r="D3" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E66" si="0" xml:space="preserve"> "/addshipment "&amp;A3&amp;" "&amp;B3&amp;" "&amp;C3&amp;" "&amp;D3</f>
+        <v>/addshipment YT8832814022182 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>230</v>
       </c>
@@ -1525,8 +1534,12 @@
       <c r="D4" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375774139249 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>231</v>
       </c>
@@ -1539,8 +1552,12 @@
       <c r="D5" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375790897557 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>232</v>
       </c>
@@ -1553,8 +1570,12 @@
       <c r="D6" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375655197242 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>233</v>
       </c>
@@ -1567,8 +1588,12 @@
       <c r="D7" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8831788528380 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>234</v>
       </c>
@@ -1581,8 +1606,12 @@
       <c r="D8" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 773401491673915 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>235</v>
       </c>
@@ -1595,8 +1624,12 @@
       <c r="D9" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78570145724720 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>236</v>
       </c>
@@ -1609,8 +1642,12 @@
       <c r="D10" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465024531980029 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>237</v>
       </c>
@@ -1623,8 +1660,12 @@
       <c r="D11" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8832747496625 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>238</v>
       </c>
@@ -1637,8 +1678,12 @@
       <c r="D12" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777374858869952 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>239</v>
       </c>
@@ -1651,8 +1696,12 @@
       <c r="D13" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375051585603 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>240</v>
       </c>
@@ -1665,8 +1714,12 @@
       <c r="D14" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465024132842895 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>241</v>
       </c>
@@ -1679,8 +1732,12 @@
       <c r="D15" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78570017584532 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>242</v>
       </c>
@@ -1693,8 +1750,12 @@
       <c r="D16" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813075241432 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>243</v>
       </c>
@@ -1707,8 +1768,12 @@
       <c r="D17" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78569798744937 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>244</v>
       </c>
@@ -1721,8 +1786,12 @@
       <c r="D18" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465026557536462 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>245</v>
       </c>
@@ -1735,8 +1804,12 @@
       <c r="D19" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813086228882 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>246</v>
       </c>
@@ -1749,8 +1822,12 @@
       <c r="D20" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813086321541 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>247</v>
       </c>
@@ -1763,8 +1840,12 @@
       <c r="D21" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777376154396721 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>248</v>
       </c>
@@ -1777,8 +1858,12 @@
       <c r="D22" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777376277668173 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>249</v>
       </c>
@@ -1791,8 +1876,12 @@
       <c r="D23" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8831570733781 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>250</v>
       </c>
@@ -1805,8 +1894,12 @@
       <c r="D24" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8833663663698 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>251</v>
       </c>
@@ -1819,8 +1912,12 @@
       <c r="D25" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777374540926514 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>252</v>
       </c>
@@ -1833,8 +1930,12 @@
       <c r="D26" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8833603282880 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>253</v>
       </c>
@@ -1847,8 +1948,12 @@
       <c r="D27" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E27" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465017164559871 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>254</v>
       </c>
@@ -1861,8 +1966,12 @@
       <c r="D28" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8833808398032 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>255</v>
       </c>
@@ -1875,8 +1984,12 @@
       <c r="D29" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78571336030299 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>256</v>
       </c>
@@ -1889,8 +2002,12 @@
       <c r="D30" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E30" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465023350363129 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>257</v>
       </c>
@@ -1903,8 +2020,12 @@
       <c r="D31" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E31" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813181118186 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>258</v>
       </c>
@@ -1917,8 +2038,12 @@
       <c r="D32" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment JT5450370100069 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>276</v>
       </c>
@@ -1931,8 +2056,12 @@
       <c r="D33" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813183000677 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>259</v>
       </c>
@@ -1945,8 +2074,12 @@
       <c r="D34" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813062922639 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>260</v>
       </c>
@@ -1959,8 +2092,12 @@
       <c r="D35" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777376302160525 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>261</v>
       </c>
@@ -1973,8 +2110,12 @@
       <c r="D36" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813184705253 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>262</v>
       </c>
@@ -1987,8 +2128,12 @@
       <c r="D37" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT883711632498 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>263</v>
       </c>
@@ -2001,8 +2146,12 @@
       <c r="D38" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment JT5450471937159 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>264</v>
       </c>
@@ -2015,8 +2164,12 @@
       <c r="D39" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment JT54500310120496 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>265</v>
       </c>
@@ -2029,8 +2182,12 @@
       <c r="D40" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E40" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 465025090790370 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>266</v>
       </c>
@@ -2043,8 +2200,12 @@
       <c r="D41" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment JT5449366764110 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>267</v>
       </c>
@@ -2057,8 +2218,12 @@
       <c r="D42" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E42" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78579817835156 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>268</v>
       </c>
@@ -2071,8 +2236,12 @@
       <c r="D43" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E43" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78570042862041 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>269</v>
       </c>
@@ -2085,8 +2254,12 @@
       <c r="D44" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E44" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777374520131651 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>270</v>
       </c>
@@ -2099,8 +2272,12 @@
       <c r="D45" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375928840521 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>271</v>
       </c>
@@ -2113,8 +2290,12 @@
       <c r="D46" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78570642085405 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>272</v>
       </c>
@@ -2127,8 +2308,12 @@
       <c r="D47" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8832681217418 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>273</v>
       </c>
@@ -2141,8 +2326,12 @@
       <c r="D48" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E48" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375160421464 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>274</v>
       </c>
@@ -2155,8 +2344,12 @@
       <c r="D49" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8832544033278 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>275</v>
       </c>
@@ -2169,8 +2362,12 @@
       <c r="D50" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E50" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813074712272 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>277</v>
       </c>
@@ -2183,8 +2380,12 @@
       <c r="D51" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777376213841768 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>278</v>
       </c>
@@ -2197,8 +2398,12 @@
       <c r="D52" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777377040759512 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>279</v>
       </c>
@@ -2211,8 +2416,12 @@
       <c r="D53" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777376280064169 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>280</v>
       </c>
@@ -2225,8 +2434,12 @@
       <c r="D54" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E54" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 7773770040744616 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>281</v>
       </c>
@@ -2239,8 +2452,12 @@
       <c r="D55" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E55" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777377040755654 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>282</v>
       </c>
@@ -2253,8 +2470,12 @@
       <c r="D56" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E56" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment JT5450363289037 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>283</v>
       </c>
@@ -2267,8 +2488,12 @@
       <c r="D57" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E57" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 777375025935966 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>284</v>
       </c>
@@ -2281,8 +2506,12 @@
       <c r="D58" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E58" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8832313297726 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>285</v>
       </c>
@@ -2295,8 +2524,12 @@
       <c r="D59" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E59" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813190869788 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>286</v>
       </c>
@@ -2309,8 +2542,12 @@
       <c r="D60" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E60" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 765038986704092 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>287</v>
       </c>
@@ -2323,8 +2560,12 @@
       <c r="D61" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E61" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8833255212688 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>288</v>
       </c>
@@ -2337,8 +2578,12 @@
       <c r="D62" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E62" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813124045375 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>289</v>
       </c>
@@ -2351,8 +2596,12 @@
       <c r="D63" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E63" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment YT8832710055318 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>290</v>
       </c>
@@ -2365,8 +2614,12 @@
       <c r="D64" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E64" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 78570135961235 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>291</v>
       </c>
@@ -2379,8 +2632,12 @@
       <c r="D65" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E65" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 250930034220114 Parviz +992937777333 Done</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>292</v>
       </c>
@@ -2393,8 +2650,12 @@
       <c r="D66" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E66" t="str">
+        <f t="shared" si="0"/>
+        <v>/addshipment 9813195681944 Zulayakho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>293</v>
       </c>
@@ -2407,8 +2668,12 @@
       <c r="D67" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E67" t="str">
+        <f t="shared" ref="E67:E130" si="1" xml:space="preserve"> "/addshipment "&amp;A67&amp;" "&amp;B67&amp;" "&amp;C67&amp;" "&amp;D67</f>
+        <v>/addshipment 777376276629734 Zulayakho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>294</v>
       </c>
@@ -2421,8 +2686,12 @@
       <c r="D68" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E68" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777375476969461 Zulayakho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>295</v>
       </c>
@@ -2435,8 +2704,12 @@
       <c r="D69" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E69" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777376405671090 Rukhshona +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>296</v>
       </c>
@@ -2449,8 +2722,12 @@
       <c r="D70" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E70" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8833795502751 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>297</v>
       </c>
@@ -2463,8 +2740,12 @@
       <c r="D71" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777376205046922 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>298</v>
       </c>
@@ -2477,8 +2758,12 @@
       <c r="D72" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465038416153185 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>299</v>
       </c>
@@ -2491,8 +2776,12 @@
       <c r="D73" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E73" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465038970739730 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>300</v>
       </c>
@@ -2505,8 +2794,12 @@
       <c r="D74" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E74" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465028414489289 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>301</v>
       </c>
@@ -2519,8 +2812,12 @@
       <c r="D75" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E75" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777376331973002 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>302</v>
       </c>
@@ -2533,8 +2830,12 @@
       <c r="D76" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777376339979471 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>303</v>
       </c>
@@ -2547,8 +2848,12 @@
       <c r="D77" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E77" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571331970631 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>304</v>
       </c>
@@ -2561,8 +2866,12 @@
       <c r="D78" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E78" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813111173537 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>305</v>
       </c>
@@ -2575,8 +2884,12 @@
       <c r="D79" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E79" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465031396850274 Abdulaminova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>306</v>
       </c>
@@ -2589,8 +2902,12 @@
       <c r="D80" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E80" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571094888265 Abdulaminova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>307</v>
       </c>
@@ -2603,8 +2920,12 @@
       <c r="D81" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E81" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465039486499124 Abdulaminova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>308</v>
       </c>
@@ -2617,8 +2938,12 @@
       <c r="D82" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E82" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450229737329 Abdulaminova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>309</v>
       </c>
@@ -2631,8 +2956,12 @@
       <c r="D83" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E83" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78570970461710 Abdulaminova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>310</v>
       </c>
@@ -2645,8 +2974,12 @@
       <c r="D84" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E84" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777375957108816 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>311</v>
       </c>
@@ -2659,8 +2992,12 @@
       <c r="D85" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E85" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT7598071748542 Gulamadsho +992947999990 Done</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>312</v>
       </c>
@@ -2673,8 +3010,12 @@
       <c r="D86" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E86" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813058590191 Gulamadsho +992947999990 Done</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>313</v>
       </c>
@@ -2687,8 +3028,12 @@
       <c r="D87" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E87" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777376121075782 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>314</v>
       </c>
@@ -2701,8 +3046,12 @@
       <c r="D88" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E88" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777375158506880 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>315</v>
       </c>
@@ -2715,8 +3064,12 @@
       <c r="D89" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E89" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5449072562285 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>316</v>
       </c>
@@ -2729,8 +3082,12 @@
       <c r="D90" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E90" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813084418656 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>317</v>
       </c>
@@ -2743,8 +3100,12 @@
       <c r="D91" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E91" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465024040019790 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>318</v>
       </c>
@@ -2757,8 +3118,12 @@
       <c r="D92" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E92" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5449389490173 Nobovar +992004664388 Done</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>319</v>
       </c>
@@ -2771,8 +3136,12 @@
       <c r="D93" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777374762490363 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>320</v>
       </c>
@@ -2785,8 +3154,12 @@
       <c r="D94" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465016643495085 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>321</v>
       </c>
@@ -2799,8 +3172,12 @@
       <c r="D95" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E95" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777374535605490 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>322</v>
       </c>
@@ -2813,8 +3190,12 @@
       <c r="D96" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E96" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465038438637883 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>323</v>
       </c>
@@ -2827,8 +3208,12 @@
       <c r="D97" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465028347127742 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>324</v>
       </c>
@@ -2841,8 +3226,12 @@
       <c r="D98" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8832856865590 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>58</v>
       </c>
@@ -2855,8 +3244,12 @@
       <c r="D99" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450422259280 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>59</v>
       </c>
@@ -2869,8 +3262,12 @@
       <c r="D100" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813174535309 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>65</v>
       </c>
@@ -2883,8 +3280,12 @@
       <c r="D101" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E101" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8834176997898 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>64</v>
       </c>
@@ -2897,8 +3298,12 @@
       <c r="D102" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E102" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571562216159 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>63</v>
       </c>
@@ -2911,8 +3316,12 @@
       <c r="D103" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E103" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450374923568 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>75</v>
       </c>
@@ -2925,8 +3334,12 @@
       <c r="D104" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E104" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813178775751 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>66</v>
       </c>
@@ -2939,8 +3352,12 @@
       <c r="D105" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E105" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571490709331 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>67</v>
       </c>
@@ -2953,8 +3370,12 @@
       <c r="D106" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E106" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5451006095978 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>68</v>
       </c>
@@ -2967,8 +3388,12 @@
       <c r="D107" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E107" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813166391765 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>66</v>
       </c>
@@ -2981,8 +3406,12 @@
       <c r="D108" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E108" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571490709331 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>60</v>
       </c>
@@ -2995,8 +3424,12 @@
       <c r="D109" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E109" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78571581576278 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>61</v>
       </c>
@@ -3009,8 +3442,12 @@
       <c r="D110" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E110" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450448286889 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>62</v>
       </c>
@@ -3023,8 +3460,12 @@
       <c r="D111" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E111" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465034893527765 Parviz +992501010400 Done</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>70</v>
       </c>
@@ -3037,8 +3478,12 @@
       <c r="D112" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E112" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8832864114554 Shuhrat +992934799393 Done</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>71</v>
       </c>
@@ -3051,8 +3496,12 @@
       <c r="D113" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E113" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777375437190940 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>74</v>
       </c>
@@ -3065,8 +3514,12 @@
       <c r="D114" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E114" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8832402363792 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>76</v>
       </c>
@@ -3079,8 +3532,12 @@
       <c r="D115" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E115" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 465025251386960 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>77</v>
       </c>
@@ -3093,8 +3550,12 @@
       <c r="D116" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E116" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813056900881 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>78</v>
       </c>
@@ -3107,8 +3568,12 @@
       <c r="D117" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E117" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT88340111116934 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>79</v>
       </c>
@@ -3121,8 +3586,12 @@
       <c r="D118" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E118" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment YT8833761536269 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>82</v>
       </c>
@@ -3135,8 +3604,12 @@
       <c r="D119" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E119" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78570044147683 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>83</v>
       </c>
@@ -3149,8 +3622,12 @@
       <c r="D120" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E120" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450732631584 Abdulamidova Zarina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>85</v>
       </c>
@@ -3163,8 +3640,12 @@
       <c r="D121" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E121" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813062347484 Rukhsora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>87</v>
       </c>
@@ -3177,8 +3658,12 @@
       <c r="D122" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E122" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813251286887 Adisa +992885084885 Done</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>90</v>
       </c>
@@ -3191,8 +3676,12 @@
       <c r="D123" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E123" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777375909488758 Sadorat +99290044044 Done</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>92</v>
       </c>
@@ -3205,8 +3694,12 @@
       <c r="D124" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E124" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450141798423 Shuhrat +992934799393 Done</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>93</v>
       </c>
@@ -3219,8 +3712,12 @@
       <c r="D125" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E125" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 78570906426799 Shuhrat +992934799393 Done</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>94</v>
       </c>
@@ -3233,8 +3730,12 @@
       <c r="D126" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E126" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450312592714 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>97</v>
       </c>
@@ -3247,8 +3748,12 @@
       <c r="D127" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E127" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777374647226454 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>98</v>
       </c>
@@ -3261,8 +3766,12 @@
       <c r="D128" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E128" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 777374547840068 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
         <v>99</v>
       </c>
@@ -3275,8 +3784,12 @@
       <c r="D129" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E129" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment 9813197866741 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
         <v>100</v>
       </c>
@@ -3289,8 +3802,12 @@
       <c r="D130" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E130" t="str">
+        <f t="shared" si="1"/>
+        <v>/addshipment JT5450473688149 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
         <v>101</v>
       </c>
@@ -3303,8 +3820,12 @@
       <c r="D131" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E131" t="str">
+        <f t="shared" ref="E131:E194" si="2" xml:space="preserve"> "/addshipment "&amp;A131&amp;" "&amp;B131&amp;" "&amp;C131&amp;" "&amp;D131</f>
+        <v>/addshipment 78571534596246 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>102</v>
       </c>
@@ -3317,8 +3838,12 @@
       <c r="D132" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E132" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571446448855 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>105</v>
       </c>
@@ -3331,8 +3856,12 @@
       <c r="D133" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E133" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8833176534856 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
         <v>106</v>
       </c>
@@ -3345,8 +3874,12 @@
       <c r="D134" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E134" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813249384816 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>107</v>
       </c>
@@ -3359,8 +3892,12 @@
       <c r="D135" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E135" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813249020347 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>108</v>
       </c>
@@ -3373,8 +3910,12 @@
       <c r="D136" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E136" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813249395827 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>109</v>
       </c>
@@ -3387,8 +3928,12 @@
       <c r="D137" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E137" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813252212417 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>110</v>
       </c>
@@ -3401,8 +3946,12 @@
       <c r="D138" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E138" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813249373652 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
         <v>111</v>
       </c>
@@ -3415,8 +3964,12 @@
       <c r="D139" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E139" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment SF1569915810605 Anvar +992501273404 Done</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
         <v>122</v>
       </c>
@@ -3429,8 +3982,12 @@
       <c r="D140" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E140" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813247828669 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>114</v>
       </c>
@@ -3443,8 +4000,12 @@
       <c r="D141" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E141" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813247798767 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>115</v>
       </c>
@@ -3457,8 +4018,12 @@
       <c r="D142" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E142" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571662603266 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>116</v>
       </c>
@@ -3471,8 +4036,12 @@
       <c r="D143" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E143" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465033835556530 Nobovar +992004664388 Done</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
         <v>119</v>
       </c>
@@ -3485,8 +4054,12 @@
       <c r="D144" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E144" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78975848342929 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
         <v>120</v>
       </c>
@@ -3499,8 +4072,12 @@
       <c r="D145" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E145" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571354016848 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
         <v>121</v>
       </c>
@@ -3513,8 +4090,12 @@
       <c r="D146" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E146" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 73622446400035 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>123</v>
       </c>
@@ -3527,8 +4108,12 @@
       <c r="D147" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E147" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813151392570 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>124</v>
       </c>
@@ -3541,8 +4126,12 @@
       <c r="D148" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E148" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT5450215217415 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
         <v>125</v>
       </c>
@@ -3555,8 +4144,12 @@
       <c r="D149" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E149" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT5450215216218 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
         <v>126</v>
       </c>
@@ -3569,8 +4162,12 @@
       <c r="D150" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E150" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT5450215215577 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
         <v>127</v>
       </c>
@@ -3583,8 +4180,12 @@
       <c r="D151" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E151" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT550215219524 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
         <v>128</v>
       </c>
@@ -3597,8 +4198,12 @@
       <c r="D152" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E152" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT550215219911 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
         <v>129</v>
       </c>
@@ -3611,8 +4216,12 @@
       <c r="D153" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E153" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT550215184829 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
         <v>130</v>
       </c>
@@ -3625,8 +4234,12 @@
       <c r="D154" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E154" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 773401956972531 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
         <v>136</v>
       </c>
@@ -3639,8 +4252,12 @@
       <c r="D155" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E155" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 777376095439151 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
         <v>131</v>
       </c>
@@ -3653,8 +4270,12 @@
       <c r="D156" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E156" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813115226398 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
         <v>132</v>
       </c>
@@ -3667,8 +4288,12 @@
       <c r="D157" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E157" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 98131534164563 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
         <v>133</v>
       </c>
@@ -3681,8 +4306,12 @@
       <c r="D158" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E158" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8832328561315 Shuhrat +992934799393 Done</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="3" t="s">
         <v>134</v>
       </c>
@@ -3695,8 +4324,12 @@
       <c r="D159" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E159" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8833194512632 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="3" t="s">
         <v>135</v>
       </c>
@@ -3709,8 +4342,12 @@
       <c r="D160" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E160" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 7857113183496 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
         <v>137</v>
       </c>
@@ -3723,8 +4360,12 @@
       <c r="D161" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E161" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 7773746621335762 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
         <v>139</v>
       </c>
@@ -3737,8 +4378,12 @@
       <c r="D162" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E162" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465046295401804 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
         <v>138</v>
       </c>
@@ -3751,8 +4396,12 @@
       <c r="D163" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E163" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465036188236337 Adisa +992885084885 Done</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
         <v>142</v>
       </c>
@@ -3765,8 +4414,12 @@
       <c r="D164" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E164" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465034660175732 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
         <v>143</v>
       </c>
@@ -3779,8 +4432,12 @@
       <c r="D165" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E165" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813024694012 Shuhrat +992934799393 Done</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
         <v>144</v>
       </c>
@@ -3793,8 +4450,12 @@
       <c r="D166" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E166" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571811440325 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
         <v>159</v>
       </c>
@@ -3807,8 +4468,12 @@
       <c r="D167" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E167" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT7599240532726 Fariza +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
         <v>145</v>
       </c>
@@ -3821,8 +4486,12 @@
       <c r="D168" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E168" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8834742974777 Fariza +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
         <v>153</v>
       </c>
@@ -3835,8 +4504,12 @@
       <c r="D169" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E169" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571470082747 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>152</v>
       </c>
@@ -3849,8 +4522,12 @@
       <c r="D170" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E170" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8834185735258 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
         <v>150</v>
       </c>
@@ -3863,8 +4540,12 @@
       <c r="D171" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E171" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78975791116210 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
         <v>147</v>
       </c>
@@ -3877,8 +4558,12 @@
       <c r="D172" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E172" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813174241255 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>148</v>
       </c>
@@ -3891,8 +4576,12 @@
       <c r="D173" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E173" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465038821488297 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="3" t="s">
         <v>149</v>
       </c>
@@ -3905,8 +4594,12 @@
       <c r="D174" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E174" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment SF1568124865380 Firdavs +992501080388 Done</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="s">
         <v>157</v>
       </c>
@@ -3919,8 +4612,12 @@
       <c r="D175" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E175" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571786774277 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="s">
         <v>151</v>
       </c>
@@ -3933,8 +4630,12 @@
       <c r="D176" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E176" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8834609191163 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
         <v>156</v>
       </c>
@@ -3947,8 +4648,12 @@
       <c r="D177" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E177" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 73622458713100 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
         <v>154</v>
       </c>
@@ -3961,8 +4666,12 @@
       <c r="D178" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E178" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571606194124 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
         <v>155</v>
       </c>
@@ -3975,8 +4684,12 @@
       <c r="D179" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E179" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 78571938507821 Munis +992554194400 Done</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
         <v>158</v>
       </c>
@@ -3989,8 +4702,12 @@
       <c r="D180" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E180" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT5450747870349 Zulaykho +992501882992 Done</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
         <v>160</v>
       </c>
@@ -4003,8 +4720,12 @@
       <c r="D181" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E181" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465034866205347 Parviz +992501010400 Done</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
         <v>161</v>
       </c>
@@ -4017,8 +4738,12 @@
       <c r="D182" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E182" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465034896107554 Parviz +992501010400 Done</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
         <v>162</v>
       </c>
@@ -4031,8 +4756,12 @@
       <c r="D183" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E183" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT9000099971508 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
         <v>163</v>
       </c>
@@ -4045,8 +4774,12 @@
       <c r="D184" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E184" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8831781361627 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
         <v>164</v>
       </c>
@@ -4059,8 +4792,12 @@
       <c r="D185" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E185" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8833836075899 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
         <v>165</v>
       </c>
@@ -4073,8 +4810,12 @@
       <c r="D186" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E186" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment JT5450620312843 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
         <v>166</v>
       </c>
@@ -4087,8 +4828,12 @@
       <c r="D187" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E187" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 773402354654336 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
         <v>167</v>
       </c>
@@ -4101,8 +4846,12 @@
       <c r="D188" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E188" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 9813177917844 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="3" t="s">
         <v>168</v>
       </c>
@@ -4115,8 +4864,12 @@
       <c r="D189" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E189" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465018892001036 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
         <v>169</v>
       </c>
@@ -4129,8 +4882,12 @@
       <c r="D190" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E190" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8832175939716 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
         <v>170</v>
       </c>
@@ -4143,8 +4900,12 @@
       <c r="D191" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E191" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465036837817921 Nodira +992501869906 Done</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
         <v>171</v>
       </c>
@@ -4157,8 +4918,12 @@
       <c r="D192" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E192" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment 465034723907022 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="3" t="s">
         <v>172</v>
       </c>
@@ -4171,8 +4936,12 @@
       <c r="D193" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E193" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8832043364202 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="3" t="s">
         <v>173</v>
       </c>
@@ -4185,8 +4954,12 @@
       <c r="D194" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E194" t="str">
+        <f t="shared" si="2"/>
+        <v>/addshipment YT8834851085373 Zokir +992933360404 Done</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
         <v>174</v>
       </c>
@@ -4199,8 +4972,12 @@
       <c r="D195" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E195" t="str">
+        <f t="shared" ref="E195:E258" si="3" xml:space="preserve"> "/addshipment "&amp;A195&amp;" "&amp;B195&amp;" "&amp;C195&amp;" "&amp;D195</f>
+        <v>/addshipment JT5449739634056 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
         <v>175</v>
       </c>
@@ -4213,8 +4990,12 @@
       <c r="D196" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E196" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8834028311124 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="3" t="s">
         <v>176</v>
       </c>
@@ -4227,8 +5008,12 @@
       <c r="D197" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E197" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 465044173979546 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>177</v>
       </c>
@@ -4241,8 +5026,12 @@
       <c r="D198" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E198" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 465017324573864 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>178</v>
       </c>
@@ -4255,8 +5044,12 @@
       <c r="D199" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E199" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8833789760510 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>179</v>
       </c>
@@ -4269,8 +5062,12 @@
       <c r="D200" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E200" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376044993809 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>180</v>
       </c>
@@ -4283,8 +5080,12 @@
       <c r="D201" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E201" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment SF5101177362237 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="3" t="s">
         <v>190</v>
       </c>
@@ -4297,8 +5098,12 @@
       <c r="D202" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E202" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8833956756412 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="3" t="s">
         <v>189</v>
       </c>
@@ -4311,8 +5116,12 @@
       <c r="D203" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E203" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376921550149 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>181</v>
       </c>
@@ -4325,8 +5134,12 @@
       <c r="D204" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E204" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8833715581394 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>183</v>
       </c>
@@ -4339,8 +5152,12 @@
       <c r="D205" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E205" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 465045674373747 Adisa +992885084885 Done</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>182</v>
       </c>
@@ -4353,8 +5170,12 @@
       <c r="D206" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E206" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813239003761 Adisa +992885084885 Done</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>183</v>
       </c>
@@ -4367,8 +5188,12 @@
       <c r="D207" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E207" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 465045674373747 Adisa +992885084885 Done</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>184</v>
       </c>
@@ -4381,8 +5206,12 @@
       <c r="D208" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E208" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777377038386312 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>185</v>
       </c>
@@ -4395,8 +5224,12 @@
       <c r="D209" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E209" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5451115651124 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>186</v>
       </c>
@@ -4409,8 +5242,12 @@
       <c r="D210" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E210" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813168906429 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>187</v>
       </c>
@@ -4423,8 +5260,12 @@
       <c r="D211" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E211" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813168081299 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>202</v>
       </c>
@@ -4437,8 +5278,12 @@
       <c r="D212" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E212" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777377115957559 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>201</v>
       </c>
@@ -4451,8 +5296,12 @@
       <c r="D213" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E213" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813236540495 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="3" t="s">
         <v>188</v>
       </c>
@@ -4465,8 +5314,12 @@
       <c r="D214" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E214" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5451459100079 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="3" t="s">
         <v>191</v>
       </c>
@@ -4479,8 +5332,12 @@
       <c r="D215" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E215" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376601392005 Khisholbegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
         <v>194</v>
       </c>
@@ -4493,8 +5350,12 @@
       <c r="D216" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E216" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376767723517 Khisholbegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="3" t="s">
         <v>195</v>
       </c>
@@ -4507,8 +5368,12 @@
       <c r="D217" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E217" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5451561011965 Khisholbegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="3" t="s">
         <v>203</v>
       </c>
@@ -4521,8 +5386,12 @@
       <c r="D218" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E218" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813222251936 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="3" t="s">
         <v>199</v>
       </c>
@@ -4535,8 +5404,12 @@
       <c r="D219" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E219" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8834393841729 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="3" t="s">
         <v>196</v>
       </c>
@@ -4549,8 +5422,12 @@
       <c r="D220" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E220" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813230744060 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="3" t="s">
         <v>197</v>
       </c>
@@ -4563,8 +5440,12 @@
       <c r="D221" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E221" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8834626103435 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="3" t="s">
         <v>204</v>
       </c>
@@ -4577,8 +5458,12 @@
       <c r="D222" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E222" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813235093085 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="3" t="s">
         <v>198</v>
       </c>
@@ -4591,8 +5476,12 @@
       <c r="D223" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E223" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376645143562 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="3" t="s">
         <v>200</v>
       </c>
@@ -4605,8 +5494,12 @@
       <c r="D224" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E224" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777376931935469 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="3" t="s">
         <v>25</v>
       </c>
@@ -4619,8 +5512,12 @@
       <c r="D225" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E225" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT883169976258 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="3" t="s">
         <v>35</v>
       </c>
@@ -4633,8 +5530,12 @@
       <c r="D226" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E226" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8831992270561 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="3" t="s">
         <v>26</v>
       </c>
@@ -4647,8 +5548,12 @@
       <c r="D227" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E227" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT3148842609075 Dilangez +992501819804 Done</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="3" t="s">
         <v>27</v>
       </c>
@@ -4661,8 +5566,12 @@
       <c r="D228" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E228" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78567501934744 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="3" t="s">
         <v>43</v>
       </c>
@@ -4675,8 +5584,12 @@
       <c r="D229" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E229" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448497039019 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="3" t="s">
         <v>28</v>
       </c>
@@ -4689,8 +5602,12 @@
       <c r="D230" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E230" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5446578048352 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="3" t="s">
         <v>31</v>
       </c>
@@ -4703,8 +5620,12 @@
       <c r="D231" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E231" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448775242977 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="3" t="s">
         <v>34</v>
       </c>
@@ -4717,8 +5638,12 @@
       <c r="D232" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E232" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5449081964836 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="3" t="s">
         <v>44</v>
       </c>
@@ -4731,8 +5656,12 @@
       <c r="D233" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E233" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448572932569 Rukhzora +992554319393 Done</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
         <v>32</v>
       </c>
@@ -4745,8 +5674,12 @@
       <c r="D234" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E234" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8831737690119 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
         <v>39</v>
       </c>
@@ -4759,8 +5692,12 @@
       <c r="D235" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E235" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777374490825535 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
         <v>40</v>
       </c>
@@ -4773,8 +5710,12 @@
       <c r="D236" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E236" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9812914971041 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
         <v>41</v>
       </c>
@@ -4787,8 +5728,12 @@
       <c r="D237" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E237" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448042527864 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="3" t="s">
         <v>42</v>
       </c>
@@ -4801,8 +5746,12 @@
       <c r="D238" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E238" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448973831585 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="3" t="s">
         <v>45</v>
       </c>
@@ -4815,8 +5764,12 @@
       <c r="D239" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E239" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8831592303427 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="3" t="s">
         <v>46</v>
       </c>
@@ -4829,8 +5782,12 @@
       <c r="D240" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E240" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8831550776450 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="3" t="s">
         <v>33</v>
       </c>
@@ -4843,8 +5800,12 @@
       <c r="D241" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E241" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT9000165918898 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="3" t="s">
         <v>36</v>
       </c>
@@ -4857,8 +5818,12 @@
       <c r="D242" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E242" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5448465081161 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="3" t="s">
         <v>37</v>
       </c>
@@ -4871,8 +5836,12 @@
       <c r="D243" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E243" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9812979415399 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="3" t="s">
         <v>38</v>
       </c>
@@ -4885,8 +5854,12 @@
       <c r="D244" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E244" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 777374086737545 Mavzuna +992994880004 Done</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="3" t="s">
         <v>47</v>
       </c>
@@ -4899,8 +5872,12 @@
       <c r="D245" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E245" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment JT5449079294979 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="3" t="s">
         <v>52</v>
       </c>
@@ -4913,8 +5890,12 @@
       <c r="D246" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E246" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78569822649320 Shifo +992909198989 Done</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="3" t="s">
         <v>48</v>
       </c>
@@ -4927,8 +5908,12 @@
       <c r="D247" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E247" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8829141445621 Sadorat +992900044044 Done</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="3" t="s">
         <v>49</v>
       </c>
@@ -4941,8 +5926,12 @@
       <c r="D248" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E248" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78567220862644 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="3" t="s">
         <v>50</v>
       </c>
@@ -4955,8 +5944,12 @@
       <c r="D249" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E249" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9812799827406 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="3" t="s">
         <v>51</v>
       </c>
@@ -4969,8 +5962,12 @@
       <c r="D250" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E250" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8830376925929 Abdulamidova Zarrina +992501922462 Done</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="3" t="s">
         <v>53</v>
       </c>
@@ -4983,8 +5980,12 @@
       <c r="D251" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E251" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78567836437685 Gulamadsho +992947999990 Done</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="3" t="s">
         <v>54</v>
       </c>
@@ -4997,8 +5998,12 @@
       <c r="D252" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E252" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9812994267990 Marbo +992501192804 Done</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="3" t="s">
         <v>55</v>
       </c>
@@ -5011,8 +6016,12 @@
       <c r="D253" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E253" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 9813009021326 Nodira +992501854049 Done</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="3" t="s">
         <v>205</v>
       </c>
@@ -5025,8 +6034,12 @@
       <c r="D254" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E254" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78572146744294 Khishobegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="3" t="s">
         <v>220</v>
       </c>
@@ -5039,8 +6052,12 @@
       <c r="D255" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E255" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 465043629465743 Khishobegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="3" t="s">
         <v>218</v>
       </c>
@@ -5053,8 +6070,12 @@
       <c r="D256" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E256" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment YT8834705575117 Khishobegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
         <v>208</v>
       </c>
@@ -5067,8 +6088,12 @@
       <c r="D257" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E257" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 78572014160566 Khishobegim +992114774111 Done</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="3" t="s">
         <v>207</v>
       </c>
@@ -5081,8 +6106,12 @@
       <c r="D258" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E258" t="str">
+        <f t="shared" si="3"/>
+        <v>/addshipment 785722261750105 Fariza +992501869996 Done</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="3" t="s">
         <v>225</v>
       </c>
@@ -5095,8 +6124,12 @@
       <c r="D259" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E259" t="str">
+        <f t="shared" ref="E259:E274" si="4" xml:space="preserve"> "/addshipment "&amp;A259&amp;" "&amp;B259&amp;" "&amp;C259&amp;" "&amp;D259</f>
+        <v>/addshipment YT8834677249546 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
         <v>214</v>
       </c>
@@ -5109,8 +6142,12 @@
       <c r="D260" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E260" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 78571964067999 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
         <v>209</v>
       </c>
@@ -5123,8 +6160,12 @@
       <c r="D261" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E261" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 78571964067986 Musso +992947940404 Done</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
         <v>210</v>
       </c>
@@ -5137,8 +6178,12 @@
       <c r="D262" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E262" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 78572534102436 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
         <v>222</v>
       </c>
@@ -5151,8 +6196,12 @@
       <c r="D263" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E263" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8834628135407 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
         <v>211</v>
       </c>
@@ -5165,8 +6214,12 @@
       <c r="D264" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E264" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 465046644758659 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
         <v>212</v>
       </c>
@@ -5179,8 +6232,12 @@
       <c r="D265" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E265" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 465046084745942 Azmina +992501049698 Done</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="3" t="s">
         <v>217</v>
       </c>
@@ -5193,8 +6250,12 @@
       <c r="D266" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E266" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8834523526548 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
         <v>216</v>
       </c>
@@ -5207,8 +6268,12 @@
       <c r="D267" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E267" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8834306048665 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="3" t="s">
         <v>213</v>
       </c>
@@ -5221,8 +6286,12 @@
       <c r="D268" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E268" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 465043636122515 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="3" t="s">
         <v>334</v>
       </c>
@@ -5235,8 +6304,12 @@
       <c r="D269" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E269" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8834523358954 Mehrona +992501661989 Done</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="3" t="s">
         <v>221</v>
       </c>
@@ -5249,8 +6322,12 @@
       <c r="D270" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E270" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 465043251866606 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="3" t="s">
         <v>215</v>
       </c>
@@ -5263,8 +6340,12 @@
       <c r="D271" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E271" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8834296229349 Shakhnoz +992111004488 Done</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="3" t="s">
         <v>219</v>
       </c>
@@ -5277,8 +6358,12 @@
       <c r="D272" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E272" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 777376128948105 Nanish +992931440994 Done</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="3" t="s">
         <v>223</v>
       </c>
@@ -5291,8 +6376,12 @@
       <c r="D273" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E273" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment YT8833942010296 Sabrina +992501143139 Done</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="3" t="s">
         <v>224</v>
       </c>
@@ -5304,6 +6393,10 @@
       </c>
       <c r="D274" t="s">
         <v>340</v>
+      </c>
+      <c r="E274" t="str">
+        <f t="shared" si="4"/>
+        <v>/addshipment 777377080321632 Zokir +992933360404 Done</v>
       </c>
     </row>
   </sheetData>

</xml_diff>